<commit_message>
feat: restore generic layout as a second embedded template set
Bring back the pre-2f7e95a generic document layout (seller block,
title top-right, labeled party block, Product/Description/Quantity/
Unit Price/Tax Rate/Line Total table, Subtotal/Tax/Total footer) as
<type>_default.xlsx for all six document types, alongside the
Tunisian "Facture" layout, now generated as <type>_tunisia.xlsx.

The Tunisia outputs are byte-identical to the previously shipped
defaults. The restored builders use their original dark header band
(newDarkHeaderStyle) since templateStyles.header was restyled for the
Tunisian layout. The default invoice also gains a Discount row and
the amount-in-words line, so an invoice with a remise still adds up.

Each template type gets its own placeholder guard test.
</commit_message>
<xml_diff>
--- a/db/templates/delivery_default.xlsx
+++ b/db/templates/delivery_default.xlsx
@@ -7,11 +7,11 @@
     <workbookView xWindow="0" yWindow="0" windowWidth="14805" windowHeight="8010"/>
   </bookViews>
   <sheets>
-    <sheet name="Bon de livraison" sheetId="1" r:id="rId1"/>
+    <sheet name="Delivery Note" sheetId="1" r:id="rId1"/>
     <sheet name="Available fields" sheetId="2" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName localSheetId="0" name="_xlnm.Print_Titles">'Bon de livraison'!$1:$11</definedName>
+    <definedName localSheetId="0" name="_xlnm.Print_Titles">'Delivery Note'!$1:$13</definedName>
   </definedNames>
   <calcPr calcId="122211"/>
 </workbook>
@@ -20,274 +20,274 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="101">
   <si>
+    <t>{{organization.name}}</t>
+  </si>
+  <si>
+    <t>{{organization.street}} {{organization.houseNumber}}</t>
+  </si>
+  <si>
+    <t>{{organization.postalCode}} {{organization.city}}</t>
+  </si>
+  <si>
+    <t>Matricule fiscal: {{organization.vatin}}</t>
+  </si>
+  <si>
+    <t>{{organization.email}} | {{organization.phone}}</t>
+  </si>
+  <si>
+    <t>DELIVERY NOTE</t>
+  </si>
+  <si>
+    <t>Delivery number: {{delivery.number}}</t>
+  </si>
+  <si>
+    <t>Delivery date: {{delivery.date}}</t>
+  </si>
+  <si>
+    <t>Order: {{delivery.orderNumber}}</t>
+  </si>
+  <si>
+    <t>Tracking number: {{delivery.trackingNumber}}</t>
+  </si>
+  <si>
+    <t>Deliver To</t>
+  </si>
+  <si>
+    <t>{{client.name}}</t>
+  </si>
+  <si>
+    <t>{{client.street}} {{client.houseNumber}}</t>
+  </si>
+  <si>
+    <t>{{client.postalCode}} {{client.city}}</t>
+  </si>
+  <si>
+    <t>Shipping address: {{delivery.shippingAddress}}</t>
+  </si>
+  <si>
+    <t>Description</t>
+  </si>
+  <si>
+    <t>Product</t>
+  </si>
+  <si>
+    <t>Quantity</t>
+  </si>
+  <si>
+    <t>{{lineItems.description}}</t>
+  </si>
+  <si>
+    <t>{{lineItems.sku}}</t>
+  </si>
+  <si>
+    <t>{{lineItems.quantity}} {{lineItems.unit}}</t>
+  </si>
+  <si>
+    <t>{{#lineItems}}</t>
+  </si>
+  <si>
+    <t>Notes: {{delivery.notes}}</t>
+  </si>
+  <si>
+    <t>Available template placeholders</t>
+  </si>
+  <si>
+    <t>Use {{placeholder}} in any cell. An unresolved one is left blank in the export, never an error.</t>
+  </si>
+  <si>
+    <t>Group</t>
+  </si>
+  <si>
+    <t>Placeholder</t>
+  </si>
+  <si>
+    <t>Header</t>
+  </si>
+  <si>
     <t>{{organization.logo}}</t>
   </si>
   <si>
-    <t>{{organization.name}}</t>
-  </si>
-  <si>
-    <t>{{organization.street}} {{organization.houseNumber}}</t>
-  </si>
-  <si>
-    <t>{{organization.postalCode}} {{organization.city}}</t>
-  </si>
-  <si>
-    <t>Tél : {{organization.phone}}</t>
-  </si>
-  <si>
-    <t>MF : {{organization.vatin}}</t>
-  </si>
-  <si>
-    <t>{{client.name}}</t>
-  </si>
-  <si>
-    <t>{{client.street}} {{client.houseNumber}}</t>
-  </si>
-  <si>
-    <t>{{client.postalCode}} {{client.city}}</t>
-  </si>
-  <si>
-    <t>Tel: {{client.phone}}</t>
-  </si>
-  <si>
-    <t>CIN: {{client.identityNumber}}</t>
-  </si>
-  <si>
-    <t>Bon de livraison N°: {{delivery.number}}</t>
-  </si>
-  <si>
-    <t>Date : {{delivery.date}}</t>
-  </si>
-  <si>
-    <t>Code</t>
-  </si>
-  <si>
-    <t>Désignation</t>
-  </si>
-  <si>
-    <t>Quantité</t>
-  </si>
-  <si>
-    <t>Unité</t>
-  </si>
-  <si>
-    <t>{{lineItems.sku}}</t>
-  </si>
-  <si>
-    <t>{{lineItems.description}}</t>
+    <t>Seller logo — place alone in a cell to anchor the uploaded image there</t>
+  </si>
+  <si>
+    <t>{{delivery.number}}</t>
+  </si>
+  <si>
+    <t>Delivery number</t>
+  </si>
+  <si>
+    <t>{{delivery.date}}</t>
+  </si>
+  <si>
+    <t>Delivery date</t>
+  </si>
+  <si>
+    <t>{{delivery.orderNumber}}</t>
+  </si>
+  <si>
+    <t>Linked order number, blank on a standalone delivery</t>
+  </si>
+  <si>
+    <t>{{delivery.shippingAddress}}</t>
+  </si>
+  <si>
+    <t>Free-text shipping address, blank if unset</t>
+  </si>
+  <si>
+    <t>{{delivery.trackingNumber}}</t>
+  </si>
+  <si>
+    <t>Tracking number, blank if unset</t>
+  </si>
+  <si>
+    <t>Seller company name</t>
+  </si>
+  <si>
+    <t>{{organization.vatin}}</t>
+  </si>
+  <si>
+    <t>Seller VAT number</t>
+  </si>
+  <si>
+    <t>{{organization.email}}</t>
+  </si>
+  <si>
+    <t>Seller email</t>
+  </si>
+  <si>
+    <t>{{organization.phone}}</t>
+  </si>
+  <si>
+    <t>Seller phone</t>
+  </si>
+  <si>
+    <t>{{organization.website}}</t>
+  </si>
+  <si>
+    <t>Seller website</t>
+  </si>
+  <si>
+    <t>{{organization.street}}</t>
+  </si>
+  <si>
+    <t>Seller street</t>
+  </si>
+  <si>
+    <t>{{organization.houseNumber}}</t>
+  </si>
+  <si>
+    <t>Seller house number</t>
+  </si>
+  <si>
+    <t>{{organization.postalCode}}</t>
+  </si>
+  <si>
+    <t>Seller postal code</t>
+  </si>
+  <si>
+    <t>{{organization.city}}</t>
+  </si>
+  <si>
+    <t>Seller city</t>
+  </si>
+  <si>
+    <t>{{organization.iban}}</t>
+  </si>
+  <si>
+    <t>Seller IBAN</t>
+  </si>
+  <si>
+    <t>{{organization.bankName}}</t>
+  </si>
+  <si>
+    <t>Seller bank name</t>
+  </si>
+  <si>
+    <t>Customer name</t>
+  </si>
+  <si>
+    <t>{{client.vatin}}</t>
+  </si>
+  <si>
+    <t>Customer VAT number</t>
+  </si>
+  <si>
+    <t>{{client.identityNumber}}</t>
+  </si>
+  <si>
+    <t>Customer national ID / CIN number</t>
+  </si>
+  <si>
+    <t>{{client.address}}</t>
+  </si>
+  <si>
+    <t>Customer single-line address</t>
+  </si>
+  <si>
+    <t>{{client.email}}</t>
+  </si>
+  <si>
+    <t>Customer email</t>
+  </si>
+  <si>
+    <t>{{client.phone}}</t>
+  </si>
+  <si>
+    <t>Customer phone</t>
+  </si>
+  <si>
+    <t>{{client.phone2}}</t>
+  </si>
+  <si>
+    <t>Customer phone 2</t>
+  </si>
+  <si>
+    <t>{{client.phone3}}</t>
+  </si>
+  <si>
+    <t>Customer phone 3</t>
+  </si>
+  <si>
+    <t>{{client.street}}</t>
+  </si>
+  <si>
+    <t>Customer street</t>
+  </si>
+  <si>
+    <t>{{client.houseNumber}}</t>
+  </si>
+  <si>
+    <t>Customer house number</t>
+  </si>
+  <si>
+    <t>{{client.postalCode}}</t>
+  </si>
+  <si>
+    <t>Customer postal code</t>
+  </si>
+  <si>
+    <t>{{client.city}}</t>
+  </si>
+  <si>
+    <t>Customer city</t>
+  </si>
+  <si>
+    <t>Item lines</t>
+  </si>
+  <si>
+    <t>Marker (not a value) — place alone in one cell of the row to repeat once per line item</t>
+  </si>
+  <si>
+    <t>Linked product's SKU</t>
+  </si>
+  <si>
+    <t>Line item description</t>
   </si>
   <si>
     <t>{{lineItems.quantity}}</t>
   </si>
   <si>
     <t>{{lineItems.unit}}</t>
-  </si>
-  <si>
-    <t>{{#lineItems}}</t>
-  </si>
-  <si>
-    <t>Cachet et Signature</t>
-  </si>
-  <si>
-    <t>IBAN : {{organization.iban}}</t>
-  </si>
-  <si>
-    <t>{{organization.bankName}}</t>
-  </si>
-  <si>
-    <t>Available template placeholders</t>
-  </si>
-  <si>
-    <t>Use {{placeholder}} in any cell. An unresolved one is left blank in the export, never an error.</t>
-  </si>
-  <si>
-    <t>Group</t>
-  </si>
-  <si>
-    <t>Placeholder</t>
-  </si>
-  <si>
-    <t>Description</t>
-  </si>
-  <si>
-    <t>Header</t>
-  </si>
-  <si>
-    <t>Seller logo — place alone in a cell to anchor the uploaded image there</t>
-  </si>
-  <si>
-    <t>{{delivery.number}}</t>
-  </si>
-  <si>
-    <t>Delivery number</t>
-  </si>
-  <si>
-    <t>{{delivery.date}}</t>
-  </si>
-  <si>
-    <t>Delivery date</t>
-  </si>
-  <si>
-    <t>{{delivery.orderNumber}}</t>
-  </si>
-  <si>
-    <t>Linked order number, blank on a standalone delivery</t>
-  </si>
-  <si>
-    <t>{{delivery.shippingAddress}}</t>
-  </si>
-  <si>
-    <t>Free-text shipping address, blank if unset</t>
-  </si>
-  <si>
-    <t>{{delivery.trackingNumber}}</t>
-  </si>
-  <si>
-    <t>Tracking number, blank if unset</t>
-  </si>
-  <si>
-    <t>Seller company name</t>
-  </si>
-  <si>
-    <t>{{organization.vatin}}</t>
-  </si>
-  <si>
-    <t>Seller VAT number</t>
-  </si>
-  <si>
-    <t>{{organization.email}}</t>
-  </si>
-  <si>
-    <t>Seller email</t>
-  </si>
-  <si>
-    <t>{{organization.phone}}</t>
-  </si>
-  <si>
-    <t>Seller phone</t>
-  </si>
-  <si>
-    <t>{{organization.website}}</t>
-  </si>
-  <si>
-    <t>Seller website</t>
-  </si>
-  <si>
-    <t>{{organization.street}}</t>
-  </si>
-  <si>
-    <t>Seller street</t>
-  </si>
-  <si>
-    <t>{{organization.houseNumber}}</t>
-  </si>
-  <si>
-    <t>Seller house number</t>
-  </si>
-  <si>
-    <t>{{organization.postalCode}}</t>
-  </si>
-  <si>
-    <t>Seller postal code</t>
-  </si>
-  <si>
-    <t>{{organization.city}}</t>
-  </si>
-  <si>
-    <t>Seller city</t>
-  </si>
-  <si>
-    <t>{{organization.iban}}</t>
-  </si>
-  <si>
-    <t>Seller IBAN</t>
-  </si>
-  <si>
-    <t>Seller bank name</t>
-  </si>
-  <si>
-    <t>Customer name</t>
-  </si>
-  <si>
-    <t>{{client.vatin}}</t>
-  </si>
-  <si>
-    <t>Customer VAT number</t>
-  </si>
-  <si>
-    <t>{{client.identityNumber}}</t>
-  </si>
-  <si>
-    <t>Customer national ID / CIN number</t>
-  </si>
-  <si>
-    <t>{{client.address}}</t>
-  </si>
-  <si>
-    <t>Customer single-line address</t>
-  </si>
-  <si>
-    <t>{{client.email}}</t>
-  </si>
-  <si>
-    <t>Customer email</t>
-  </si>
-  <si>
-    <t>{{client.phone}}</t>
-  </si>
-  <si>
-    <t>Customer phone</t>
-  </si>
-  <si>
-    <t>{{client.phone2}}</t>
-  </si>
-  <si>
-    <t>Customer phone 2</t>
-  </si>
-  <si>
-    <t>{{client.phone3}}</t>
-  </si>
-  <si>
-    <t>Customer phone 3</t>
-  </si>
-  <si>
-    <t>{{client.street}}</t>
-  </si>
-  <si>
-    <t>Customer street</t>
-  </si>
-  <si>
-    <t>{{client.houseNumber}}</t>
-  </si>
-  <si>
-    <t>Customer house number</t>
-  </si>
-  <si>
-    <t>{{client.postalCode}}</t>
-  </si>
-  <si>
-    <t>Customer postal code</t>
-  </si>
-  <si>
-    <t>{{client.city}}</t>
-  </si>
-  <si>
-    <t>Customer city</t>
-  </si>
-  <si>
-    <t>Item lines</t>
-  </si>
-  <si>
-    <t>Marker (not a value) — place alone in one cell of the row to repeat once per line item</t>
-  </si>
-  <si>
-    <t>Linked product's SKU</t>
-  </si>
-  <si>
-    <t>Line item description</t>
-  </si>
-  <si>
-    <t>Quantity</t>
   </si>
   <si>
     <t>Unit of measure, blank if unset</t>
@@ -354,13 +354,13 @@
     <font>
       <family val="2"/>
       <b val="1"/>
-      <color/>
-      <sz val="14"/>
+      <color rgb="FFFFFFFF"/>
     </font>
     <font>
       <family val="2"/>
       <b val="1"/>
-      <color rgb="FFFFFFFF"/>
+      <color/>
+      <sz val="14"/>
     </font>
     <font>
       <family val="2"/>
@@ -412,7 +412,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="true" applyAlignment="false">
       <alignment/>
@@ -438,10 +438,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyAlignment="false">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="true" applyFill="true" applyAlignment="true">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyAlignment="false">
       <alignment/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="true" applyFill="true" applyAlignment="false">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="true" applyFill="true" applyAlignment="false">
       <alignment/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="true" applyFill="true" applyAlignment="false">
@@ -723,149 +726,112 @@
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col customWidth="true" max="1" min="1" width="14"/>
-    <col customWidth="true" max="2" min="2" width="34"/>
-    <col customWidth="true" max="4" min="3" width="16"/>
+    <col customWidth="true" max="1" min="1" width="24"/>
+    <col customWidth="true" max="2" min="2" width="16"/>
+    <col customWidth="true" max="3" min="3" width="22"/>
+    <col customWidth="true" max="4" min="4" width="16"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="7" t="s">
+      <c r="E1" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s">
+        <v>1</v>
+      </c>
+      <c r="E2" t="s">
         <v>6</v>
       </c>
-      <c r="D1" s="7"/>
-      <c r="E1" s="7"/>
-      <c r="F1" s="7"/>
-    </row>
-    <row r="2">
-      <c r="C2" s="7" t="s">
+    </row>
+    <row r="3">
+      <c r="A3" t="s">
+        <v>2</v>
+      </c>
+      <c r="E3" t="s">
         <v>7</v>
       </c>
-      <c r="D2" s="7"/>
-      <c r="E2" s="7"/>
-      <c r="F2" s="7"/>
-    </row>
-    <row r="3">
-      <c r="A3" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C3" s="7" t="s">
-        <v>8</v>
-      </c>
-      <c r="D3" s="7"/>
-      <c r="E3" s="7"/>
-      <c r="F3" s="7"/>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>2</v>
-      </c>
-      <c r="C4" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="D4" s="7"/>
-      <c r="E4" s="7"/>
-      <c r="F4" s="7"/>
+        <v>3</v>
+      </c>
+      <c r="E4" t="s">
+        <v>8</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>3</v>
-      </c>
-      <c r="C5" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="E5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="D5" s="7"/>
-      <c r="E5" s="7"/>
-      <c r="F5" s="7"/>
-    </row>
-    <row r="6">
-      <c r="A6" t="s">
-        <v>4</v>
-      </c>
-      <c r="C6" s="7"/>
-      <c r="D6" s="7"/>
-      <c r="E6" s="7"/>
-      <c r="F6" s="7"/>
-    </row>
-    <row r="7">
-      <c r="A7" t="s">
-        <v>5</v>
-      </c>
     </row>
     <row r="8">
-      <c r="C8" s="7" t="s">
+      <c r="A8" t="s">
         <v>11</v>
       </c>
-      <c r="D8" s="7"/>
-      <c r="E8" s="7"/>
-      <c r="F8" s="7"/>
     </row>
     <row r="9">
-      <c r="C9" s="7"/>
-      <c r="D9" s="7" t="s">
+      <c r="A9" t="s">
         <v>12</v>
       </c>
-      <c r="E9" s="7"/>
-      <c r="F9" s="7"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="11">
-      <c r="A11" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="B11" s="4" t="s">
+      <c r="A11" t="s">
         <v>14</v>
       </c>
-      <c r="C11" s="4" t="s">
+    </row>
+    <row r="13">
+      <c r="A13" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="D11" s="4" t="s">
+      <c r="B13" s="9"/>
+      <c r="C13" s="9" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="7" t="s">
+      <c r="D13" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="B12" s="7" t="s">
+    </row>
+    <row r="14">
+      <c r="A14" t="s">
         <v>18</v>
       </c>
-      <c r="C12" s="5" t="s">
+      <c r="C14" t="s">
         <v>19</v>
       </c>
-      <c r="D12" s="7" t="s">
+      <c r="D14" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="J12" t="s">
+      <c r="E14" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="18">
-      <c r="D18" s="8" t="s">
+      <c r="A18" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" t="s">
-        <v>23</v>
-      </c>
-      <c r="D22" t="s">
-        <v>24</v>
-      </c>
-    </row>
   </sheetData>
-  <mergeCells count="10">
-    <mergeCell ref="C1:F1"/>
-    <mergeCell ref="C2:F2"/>
-    <mergeCell ref="C3:F3"/>
-    <mergeCell ref="C4:F4"/>
-    <mergeCell ref="C5:F5"/>
-    <mergeCell ref="C8:F8"/>
-    <mergeCell ref="D9:F9"/>
-    <mergeCell ref="D18:G18"/>
-    <mergeCell ref="A22:C22"/>
-    <mergeCell ref="D22:G22"/>
+  <mergeCells count="2">
+    <mergeCell ref="A13:B13"/>
+    <mergeCell ref="A14:B14"/>
   </mergeCells>
   <pageSetup fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
@@ -885,266 +851,266 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="9" t="s">
+      <c r="A1" s="10" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="13" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="11" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="12" t="s">
+      <c r="B4" s="11" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="10" t="s">
+      <c r="C4" s="11" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="12" t="s">
         <v>27</v>
-      </c>
-      <c r="B4" s="10" t="s">
-        <v>28</v>
-      </c>
-      <c r="C4" s="10" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="11" t="s">
-        <v>30</v>
       </c>
     </row>
     <row r="6">
       <c r="B6" t="s">
-        <v>0</v>
+        <v>28</v>
       </c>
       <c r="C6" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
     </row>
     <row r="7">
       <c r="B7" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="C7" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
     </row>
     <row r="8">
       <c r="B8" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C8" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="9">
       <c r="B9" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="C9" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
     </row>
     <row r="10">
       <c r="B10" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="C10" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
     </row>
     <row r="11">
       <c r="B11" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C11" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
     </row>
     <row r="12">
       <c r="B12" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C12" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
     </row>
     <row r="13">
       <c r="B13" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C13" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
     </row>
     <row r="14">
       <c r="B14" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="C14" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
     </row>
     <row r="15">
       <c r="B15" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="C15" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
     </row>
     <row r="16">
       <c r="B16" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="C16" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="17">
       <c r="B17" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="C17" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="18">
       <c r="B18" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="C18" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
     </row>
     <row r="19">
       <c r="B19" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="C19" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
     </row>
     <row r="20">
       <c r="B20" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="C20" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
     </row>
     <row r="21">
       <c r="B21" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="C21" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
     </row>
     <row r="22">
       <c r="B22" t="s">
-        <v>24</v>
+        <v>59</v>
       </c>
       <c r="C22" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="23">
       <c r="B23" t="s">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="C23" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="24">
       <c r="B24" t="s">
+        <v>62</v>
+      </c>
+      <c r="C24" t="s">
         <v>63</v>
-      </c>
-      <c r="C24" t="s">
-        <v>64</v>
       </c>
     </row>
     <row r="25">
       <c r="B25" t="s">
+        <v>64</v>
+      </c>
+      <c r="C25" t="s">
         <v>65</v>
-      </c>
-      <c r="C25" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="26">
       <c r="B26" t="s">
+        <v>66</v>
+      </c>
+      <c r="C26" t="s">
         <v>67</v>
-      </c>
-      <c r="C26" t="s">
-        <v>68</v>
       </c>
     </row>
     <row r="27">
       <c r="B27" t="s">
+        <v>68</v>
+      </c>
+      <c r="C27" t="s">
         <v>69</v>
-      </c>
-      <c r="C27" t="s">
-        <v>70</v>
       </c>
     </row>
     <row r="28">
       <c r="B28" t="s">
+        <v>70</v>
+      </c>
+      <c r="C28" t="s">
         <v>71</v>
-      </c>
-      <c r="C28" t="s">
-        <v>72</v>
       </c>
     </row>
     <row r="29">
       <c r="B29" t="s">
+        <v>72</v>
+      </c>
+      <c r="C29" t="s">
         <v>73</v>
-      </c>
-      <c r="C29" t="s">
-        <v>74</v>
       </c>
     </row>
     <row r="30">
       <c r="B30" t="s">
+        <v>74</v>
+      </c>
+      <c r="C30" t="s">
         <v>75</v>
-      </c>
-      <c r="C30" t="s">
-        <v>76</v>
       </c>
     </row>
     <row r="31">
       <c r="B31" t="s">
+        <v>76</v>
+      </c>
+      <c r="C31" t="s">
         <v>77</v>
-      </c>
-      <c r="C31" t="s">
-        <v>78</v>
       </c>
     </row>
     <row r="32">
       <c r="B32" t="s">
+        <v>78</v>
+      </c>
+      <c r="C32" t="s">
         <v>79</v>
-      </c>
-      <c r="C32" t="s">
-        <v>80</v>
       </c>
     </row>
     <row r="33">
       <c r="B33" t="s">
+        <v>80</v>
+      </c>
+      <c r="C33" t="s">
         <v>81</v>
-      </c>
-      <c r="C33" t="s">
-        <v>82</v>
       </c>
     </row>
     <row r="34">
       <c r="B34" t="s">
+        <v>82</v>
+      </c>
+      <c r="C34" t="s">
         <v>83</v>
       </c>
-      <c r="C34" t="s">
+    </row>
+    <row r="35">
+      <c r="A35" s="12" t="s">
         <v>84</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="11" t="s">
-        <v>85</v>
       </c>
     </row>
     <row r="36">
@@ -1152,15 +1118,15 @@
         <v>21</v>
       </c>
       <c r="C36" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="37">
       <c r="B37" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="C37" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="38">
@@ -1168,27 +1134,27 @@
         <v>18</v>
       </c>
       <c r="C38" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="39">
       <c r="B39" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="C39" t="s">
-        <v>89</v>
+        <v>17</v>
       </c>
     </row>
     <row r="40">
       <c r="B40" t="s">
-        <v>20</v>
+        <v>89</v>
       </c>
       <c r="C40" t="s">
         <v>90</v>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="11" t="s">
+      <c r="A41" s="12" t="s">
         <v>91</v>
       </c>
     </row>
@@ -1201,7 +1167,7 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="11" t="s">
+      <c r="A43" s="12" t="s">
         <v>94</v>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: print every client's address line on documents
The Tunisia invoice printed only the Cash Book's free-text address, and
every other client layout only the street, so one kind of client always
got a blank line. A computed {{client.addressLine}} prints the street
and house number, else the free-text address, in all six layouts.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/db/templates/delivery_default.xlsx
+++ b/db/templates/delivery_default.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="101">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="102">
   <si>
     <t>{{organization.name}}</t>
   </si>
@@ -56,7 +56,7 @@
     <t>{{client.name}}</t>
   </si>
   <si>
-    <t>{{client.street}} {{client.houseNumber}}</t>
+    <t>{{client.addressLine}}</t>
   </si>
   <si>
     <t>{{client.postalCode}} {{client.city}}</t>
@@ -222,6 +222,9 @@
   </si>
   <si>
     <t>Customer single-line address</t>
+  </si>
+  <si>
+    <t>Customer street and house number, or the single-line address when there is no street</t>
   </si>
   <si>
     <t>{{client.email}}</t>
@@ -1046,84 +1049,84 @@
     </row>
     <row r="27">
       <c r="B27" t="s">
+        <v>12</v>
+      </c>
+      <c r="C27" t="s">
         <v>68</v>
-      </c>
-      <c r="C27" t="s">
-        <v>69</v>
       </c>
     </row>
     <row r="28">
       <c r="B28" t="s">
+        <v>69</v>
+      </c>
+      <c r="C28" t="s">
         <v>70</v>
-      </c>
-      <c r="C28" t="s">
-        <v>71</v>
       </c>
     </row>
     <row r="29">
       <c r="B29" t="s">
+        <v>71</v>
+      </c>
+      <c r="C29" t="s">
         <v>72</v>
-      </c>
-      <c r="C29" t="s">
-        <v>73</v>
       </c>
     </row>
     <row r="30">
       <c r="B30" t="s">
+        <v>73</v>
+      </c>
+      <c r="C30" t="s">
         <v>74</v>
-      </c>
-      <c r="C30" t="s">
-        <v>75</v>
       </c>
     </row>
     <row r="31">
       <c r="B31" t="s">
+        <v>75</v>
+      </c>
+      <c r="C31" t="s">
         <v>76</v>
-      </c>
-      <c r="C31" t="s">
-        <v>77</v>
       </c>
     </row>
     <row r="32">
       <c r="B32" t="s">
+        <v>77</v>
+      </c>
+      <c r="C32" t="s">
         <v>78</v>
-      </c>
-      <c r="C32" t="s">
-        <v>79</v>
       </c>
     </row>
     <row r="33">
       <c r="B33" t="s">
+        <v>79</v>
+      </c>
+      <c r="C33" t="s">
         <v>80</v>
-      </c>
-      <c r="C33" t="s">
-        <v>81</v>
       </c>
     </row>
     <row r="34">
       <c r="B34" t="s">
+        <v>81</v>
+      </c>
+      <c r="C34" t="s">
         <v>82</v>
       </c>
-      <c r="C34" t="s">
+    </row>
+    <row r="35">
+      <c r="B35" t="s">
         <v>83</v>
       </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="12" t="s">
+      <c r="C35" t="s">
         <v>84</v>
       </c>
     </row>
     <row r="36">
-      <c r="B36" t="s">
-        <v>21</v>
-      </c>
-      <c r="C36" t="s">
+      <c r="A36" s="12" t="s">
         <v>85</v>
       </c>
     </row>
     <row r="37">
       <c r="B37" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="C37" t="s">
         <v>86</v>
@@ -1131,7 +1134,7 @@
     </row>
     <row r="38">
       <c r="B38" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C38" t="s">
         <v>87</v>
@@ -1139,10 +1142,10 @@
     </row>
     <row r="39">
       <c r="B39" t="s">
+        <v>18</v>
+      </c>
+      <c r="C39" t="s">
         <v>88</v>
-      </c>
-      <c r="C39" t="s">
-        <v>17</v>
       </c>
     </row>
     <row r="40">
@@ -1150,58 +1153,66 @@
         <v>89</v>
       </c>
       <c r="C40" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="B41" t="s">
         <v>90</v>
       </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="12" t="s">
+      <c r="C41" t="s">
         <v>91</v>
       </c>
     </row>
     <row r="42">
-      <c r="B42" t="s">
+      <c r="A42" s="12" t="s">
         <v>92</v>
       </c>
-      <c r="C42" t="s">
+    </row>
+    <row r="43">
+      <c r="B43" t="s">
         <v>93</v>
       </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="12" t="s">
+      <c r="C43" t="s">
         <v>94</v>
       </c>
     </row>
     <row r="44">
-      <c r="B44" t="s">
+      <c r="A44" s="12" t="s">
         <v>95</v>
-      </c>
-      <c r="C44" t="s">
-        <v>96</v>
       </c>
     </row>
     <row r="45">
       <c r="B45" t="s">
+        <v>96</v>
+      </c>
+      <c r="C45" t="s">
         <v>97</v>
-      </c>
-      <c r="C45" t="s">
-        <v>98</v>
       </c>
     </row>
     <row r="46">
       <c r="B46" t="s">
+        <v>98</v>
+      </c>
+      <c r="C46" t="s">
         <v>99</v>
       </c>
-      <c r="C46" t="s">
+    </row>
+    <row r="47">
+      <c r="B47" t="s">
         <v>100</v>
+      </c>
+      <c r="C47" t="s">
+        <v>101</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="5">
     <mergeCell ref="A2:C2"/>
     <mergeCell ref="A5:C5"/>
-    <mergeCell ref="A35:C35"/>
-    <mergeCell ref="A41:C41"/>
-    <mergeCell ref="A43:C43"/>
+    <mergeCell ref="A36:C36"/>
+    <mergeCell ref="A42:C42"/>
+    <mergeCell ref="A44:C44"/>
   </mergeCells>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix: print every client's address line on documents (#539)
The Tunisia invoice printed only the Cash Book's free-text address, and
every other client layout only the street, so one kind of client always
got a blank line. A computed {{client.addressLine}} prints the street
and house number, else the free-text address, in all six layouts.

Co-authored-by: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/db/templates/delivery_default.xlsx
+++ b/db/templates/delivery_default.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="101">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="102">
   <si>
     <t>{{organization.name}}</t>
   </si>
@@ -56,7 +56,7 @@
     <t>{{client.name}}</t>
   </si>
   <si>
-    <t>{{client.street}} {{client.houseNumber}}</t>
+    <t>{{client.addressLine}}</t>
   </si>
   <si>
     <t>{{client.postalCode}} {{client.city}}</t>
@@ -222,6 +222,9 @@
   </si>
   <si>
     <t>Customer single-line address</t>
+  </si>
+  <si>
+    <t>Customer street and house number, or the single-line address when there is no street</t>
   </si>
   <si>
     <t>{{client.email}}</t>
@@ -1046,84 +1049,84 @@
     </row>
     <row r="27">
       <c r="B27" t="s">
+        <v>12</v>
+      </c>
+      <c r="C27" t="s">
         <v>68</v>
-      </c>
-      <c r="C27" t="s">
-        <v>69</v>
       </c>
     </row>
     <row r="28">
       <c r="B28" t="s">
+        <v>69</v>
+      </c>
+      <c r="C28" t="s">
         <v>70</v>
-      </c>
-      <c r="C28" t="s">
-        <v>71</v>
       </c>
     </row>
     <row r="29">
       <c r="B29" t="s">
+        <v>71</v>
+      </c>
+      <c r="C29" t="s">
         <v>72</v>
-      </c>
-      <c r="C29" t="s">
-        <v>73</v>
       </c>
     </row>
     <row r="30">
       <c r="B30" t="s">
+        <v>73</v>
+      </c>
+      <c r="C30" t="s">
         <v>74</v>
-      </c>
-      <c r="C30" t="s">
-        <v>75</v>
       </c>
     </row>
     <row r="31">
       <c r="B31" t="s">
+        <v>75</v>
+      </c>
+      <c r="C31" t="s">
         <v>76</v>
-      </c>
-      <c r="C31" t="s">
-        <v>77</v>
       </c>
     </row>
     <row r="32">
       <c r="B32" t="s">
+        <v>77</v>
+      </c>
+      <c r="C32" t="s">
         <v>78</v>
-      </c>
-      <c r="C32" t="s">
-        <v>79</v>
       </c>
     </row>
     <row r="33">
       <c r="B33" t="s">
+        <v>79</v>
+      </c>
+      <c r="C33" t="s">
         <v>80</v>
-      </c>
-      <c r="C33" t="s">
-        <v>81</v>
       </c>
     </row>
     <row r="34">
       <c r="B34" t="s">
+        <v>81</v>
+      </c>
+      <c r="C34" t="s">
         <v>82</v>
       </c>
-      <c r="C34" t="s">
+    </row>
+    <row r="35">
+      <c r="B35" t="s">
         <v>83</v>
       </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="12" t="s">
+      <c r="C35" t="s">
         <v>84</v>
       </c>
     </row>
     <row r="36">
-      <c r="B36" t="s">
-        <v>21</v>
-      </c>
-      <c r="C36" t="s">
+      <c r="A36" s="12" t="s">
         <v>85</v>
       </c>
     </row>
     <row r="37">
       <c r="B37" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="C37" t="s">
         <v>86</v>
@@ -1131,7 +1134,7 @@
     </row>
     <row r="38">
       <c r="B38" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C38" t="s">
         <v>87</v>
@@ -1139,10 +1142,10 @@
     </row>
     <row r="39">
       <c r="B39" t="s">
+        <v>18</v>
+      </c>
+      <c r="C39" t="s">
         <v>88</v>
-      </c>
-      <c r="C39" t="s">
-        <v>17</v>
       </c>
     </row>
     <row r="40">
@@ -1150,58 +1153,66 @@
         <v>89</v>
       </c>
       <c r="C40" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="B41" t="s">
         <v>90</v>
       </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="12" t="s">
+      <c r="C41" t="s">
         <v>91</v>
       </c>
     </row>
     <row r="42">
-      <c r="B42" t="s">
+      <c r="A42" s="12" t="s">
         <v>92</v>
       </c>
-      <c r="C42" t="s">
+    </row>
+    <row r="43">
+      <c r="B43" t="s">
         <v>93</v>
       </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="12" t="s">
+      <c r="C43" t="s">
         <v>94</v>
       </c>
     </row>
     <row r="44">
-      <c r="B44" t="s">
+      <c r="A44" s="12" t="s">
         <v>95</v>
-      </c>
-      <c r="C44" t="s">
-        <v>96</v>
       </c>
     </row>
     <row r="45">
       <c r="B45" t="s">
+        <v>96</v>
+      </c>
+      <c r="C45" t="s">
         <v>97</v>
-      </c>
-      <c r="C45" t="s">
-        <v>98</v>
       </c>
     </row>
     <row r="46">
       <c r="B46" t="s">
+        <v>98</v>
+      </c>
+      <c r="C46" t="s">
         <v>99</v>
       </c>
-      <c r="C46" t="s">
+    </row>
+    <row r="47">
+      <c r="B47" t="s">
         <v>100</v>
+      </c>
+      <c r="C47" t="s">
+        <v>101</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="5">
     <mergeCell ref="A2:C2"/>
     <mergeCell ref="A5:C5"/>
-    <mergeCell ref="A35:C35"/>
-    <mergeCell ref="A41:C41"/>
-    <mergeCell ref="A43:C43"/>
+    <mergeCell ref="A36:C36"/>
+    <mergeCell ref="A42:C42"/>
+    <mergeCell ref="A44:C44"/>
   </mergeCells>
 </worksheet>
 </file>
</xml_diff>